<commit_message>
Champions hub: interdependent filters, reset button, tier-ranked default order, and Next title column
Filters (scope/sport/region) now offer only options available under the others; dedicated Reset clears filters and sort. Competitions default-ordered by the workbook My Tier Rank (lowest first, not shown). New sortable Next title column from the Next Awarded year. Build script and Championship type carry tier + nextAwarded.
</commit_message>
<xml_diff>
--- a/ZoneZero_Champions.xlsx
+++ b/ZoneZero_Champions.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashwi\Desktop\Projects\Metro Area Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D451B1E6-C1E1-4417-93AD-E2841FBFDF47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{302CC4B3-1AA4-4950-8B66-61A0F49D6AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3750" yWindow="510" windowWidth="26940" windowHeight="16725" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16140" yWindow="555" windowWidth="26940" windowHeight="16725" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$75</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="173">
   <si>
     <t>Sport</t>
   </si>
@@ -549,6 +552,9 @@
   </si>
   <si>
     <t>Olympic women's basketball</t>
+  </si>
+  <si>
+    <t>My Tier Rank</t>
   </si>
 </sst>
 </file>
@@ -929,7 +935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
@@ -938,10 +944,10 @@
     <col min="5" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -966,1492 +972,1718 @@
       <c r="H1" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2">
+        <v>2022</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2">
+        <v>2026</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3">
+        <v>2024</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3">
+        <v>2028</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>73</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>74</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C4" t="s">
         <v>75</v>
-      </c>
-      <c r="D2">
-        <v>2025</v>
-      </c>
-      <c r="G2" t="s">
-        <v>40</v>
-      </c>
-      <c r="H2">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3">
-        <v>2025</v>
-      </c>
-      <c r="G3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H3">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" t="s">
-        <v>69</v>
       </c>
       <c r="D4">
         <v>2025</v>
       </c>
       <c r="G4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4">
+        <v>2026</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
         <v>13</v>
       </c>
-      <c r="H4">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5" t="s">
-        <v>61</v>
-      </c>
       <c r="D5">
-        <v>2025</v>
-      </c>
-      <c r="G5" t="s">
-        <v>40</v>
+        <v>2023</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
       </c>
       <c r="H5">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>133</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>134</v>
       </c>
       <c r="D6">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G6" t="s">
-        <v>64</v>
+        <v>135</v>
       </c>
       <c r="H6">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>149</v>
+        <v>81</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>82</v>
       </c>
       <c r="D7">
-        <v>2025</v>
-      </c>
-      <c r="G7" t="s">
-        <v>40</v>
+        <v>2026</v>
+      </c>
+      <c r="F7" t="s">
+        <v>38</v>
       </c>
       <c r="H7">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C8" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="D8">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="G8" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="H8">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>90</v>
       </c>
       <c r="D9">
-        <v>2022</v>
-      </c>
-      <c r="E9" t="s">
-        <v>10</v>
+        <v>2026</v>
+      </c>
+      <c r="G9" t="s">
+        <v>19</v>
       </c>
       <c r="H9">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="D10">
+        <v>2024</v>
+      </c>
+      <c r="E10" t="s">
+        <v>38</v>
+      </c>
+      <c r="H10">
+        <v>2028</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C11" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11">
+        <v>2026</v>
+      </c>
+      <c r="E11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>2030</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12">
         <v>2025</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G12" t="s">
         <v>40</v>
       </c>
-      <c r="H10">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" t="s">
-        <v>155</v>
-      </c>
-      <c r="C11" t="s">
-        <v>159</v>
-      </c>
-      <c r="D11">
-        <v>2025</v>
-      </c>
-      <c r="E11" t="s">
-        <v>36</v>
-      </c>
-      <c r="H11">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s">
-        <v>160</v>
-      </c>
-      <c r="C12" t="s">
-        <v>161</v>
-      </c>
-      <c r="D12">
-        <v>2026</v>
-      </c>
-      <c r="G12" t="s">
-        <v>51</v>
-      </c>
       <c r="H12">
         <v>2026</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="B13" t="s">
-        <v>162</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="D13">
         <v>2025</v>
       </c>
       <c r="G13" t="s">
-        <v>164</v>
+        <v>13</v>
       </c>
       <c r="H13">
         <v>2026</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14">
+        <v>2025</v>
+      </c>
+      <c r="G14" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14">
+        <v>2026</v>
+      </c>
+      <c r="I14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" t="s">
+        <v>114</v>
+      </c>
+      <c r="D15">
+        <v>2026</v>
+      </c>
+      <c r="G15" t="s">
+        <v>40</v>
+      </c>
+      <c r="H15">
+        <v>2027</v>
+      </c>
+      <c r="I15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B14" t="s">
-        <v>165</v>
-      </c>
-      <c r="C14" t="s">
-        <v>163</v>
-      </c>
-      <c r="D14">
-        <v>2026</v>
-      </c>
-      <c r="G14" t="s">
-        <v>16</v>
-      </c>
-      <c r="H14">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15">
-        <v>2021</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="B16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16">
+        <v>2026</v>
+      </c>
+      <c r="F16" t="s">
+        <v>33</v>
+      </c>
+      <c r="H16">
+        <v>2027</v>
+      </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17">
+        <v>2026</v>
+      </c>
+      <c r="G17" t="s">
+        <v>72</v>
+      </c>
+      <c r="H17">
+        <v>2027</v>
+      </c>
+      <c r="I17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18">
+        <v>2026</v>
+      </c>
+      <c r="G18" t="s">
+        <v>22</v>
+      </c>
+      <c r="H18">
+        <v>2027</v>
+      </c>
+      <c r="I18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" t="s">
+        <v>82</v>
+      </c>
+      <c r="D19">
+        <v>2026</v>
+      </c>
+      <c r="G19" t="s">
+        <v>47</v>
+      </c>
+      <c r="H19">
+        <v>2027</v>
+      </c>
+      <c r="I19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>127</v>
+      </c>
+      <c r="C20" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20">
+        <v>2026</v>
+      </c>
+      <c r="G20" t="s">
+        <v>40</v>
+      </c>
+      <c r="H20">
+        <v>2027</v>
+      </c>
+      <c r="I20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21">
+        <v>2023</v>
+      </c>
+      <c r="E21" t="s">
         <v>10</v>
       </c>
-      <c r="H15">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" t="s">
-        <v>65</v>
-      </c>
-      <c r="C16" t="s">
-        <v>66</v>
-      </c>
-      <c r="D16">
-        <v>2025</v>
-      </c>
-      <c r="G16" t="s">
-        <v>13</v>
-      </c>
-      <c r="H16">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" t="s">
-        <v>146</v>
-      </c>
-      <c r="C17" t="s">
-        <v>147</v>
-      </c>
-      <c r="D17">
-        <v>2025</v>
-      </c>
-      <c r="G17" t="s">
-        <v>56</v>
-      </c>
-      <c r="H17">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>122</v>
-      </c>
-      <c r="B18" t="s">
-        <v>57</v>
-      </c>
-      <c r="C18" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18">
-        <v>2025</v>
-      </c>
-      <c r="G18" t="s">
-        <v>40</v>
-      </c>
-      <c r="H18">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="H21">
+        <v>2027</v>
+      </c>
+      <c r="I21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>17</v>
       </c>
-      <c r="B19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19">
-        <v>2025</v>
-      </c>
-      <c r="G19" t="s">
-        <v>40</v>
-      </c>
-      <c r="H19">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" t="s">
-        <v>22</v>
-      </c>
-      <c r="D20">
+      <c r="B22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22">
         <v>2023</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E22" t="s">
         <v>10</v>
       </c>
-      <c r="H20">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>113</v>
-      </c>
-      <c r="C21" t="s">
-        <v>114</v>
-      </c>
-      <c r="D21">
-        <v>2026</v>
-      </c>
-      <c r="G21" t="s">
-        <v>40</v>
-      </c>
-      <c r="H21">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" t="s">
-        <v>115</v>
-      </c>
-      <c r="C22" t="s">
-        <v>116</v>
-      </c>
-      <c r="D22">
-        <v>2026</v>
-      </c>
-      <c r="G22" t="s">
-        <v>40</v>
-      </c>
       <c r="H22">
         <v>2027</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="C23" t="s">
-        <v>118</v>
+        <v>40</v>
       </c>
       <c r="D23">
-        <v>2026</v>
-      </c>
-      <c r="F23" t="s">
-        <v>38</v>
+        <v>2024</v>
+      </c>
+      <c r="E23" t="s">
+        <v>10</v>
       </c>
       <c r="H23">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2028</v>
+      </c>
+      <c r="I23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B24" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="C24" t="s">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="D24">
-        <v>2026</v>
-      </c>
-      <c r="G24" t="s">
-        <v>121</v>
+        <v>2024</v>
+      </c>
+      <c r="E24" t="s">
+        <v>33</v>
       </c>
       <c r="H24">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2028</v>
+      </c>
+      <c r="I24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="B25" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="C25" t="s">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="D25">
-        <v>2023</v>
-      </c>
-      <c r="E25" t="s">
-        <v>10</v>
+        <v>2025</v>
+      </c>
+      <c r="G25" t="s">
+        <v>64</v>
       </c>
       <c r="H25">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2026</v>
+      </c>
+      <c r="I25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
-        <v>25</v>
+        <v>155</v>
       </c>
       <c r="C26" t="s">
-        <v>28</v>
+        <v>159</v>
       </c>
       <c r="D26">
         <v>2025</v>
       </c>
       <c r="E26" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="H26">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2026</v>
+      </c>
+      <c r="I26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>133</v>
+        <v>160</v>
       </c>
       <c r="C27" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="D27">
         <v>2026</v>
       </c>
       <c r="G27" t="s">
-        <v>135</v>
+        <v>51</v>
       </c>
       <c r="H27">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2026</v>
+      </c>
+      <c r="I27">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>162</v>
       </c>
       <c r="C28" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="D28">
-        <v>2024</v>
-      </c>
-      <c r="E28" t="s">
-        <v>31</v>
+        <v>2025</v>
+      </c>
+      <c r="G28" t="s">
+        <v>164</v>
       </c>
       <c r="H28">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2026</v>
+      </c>
+      <c r="I28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>14</v>
       </c>
       <c r="B29" t="s">
-        <v>50</v>
+        <v>165</v>
       </c>
       <c r="C29" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="D29">
+        <v>2026</v>
+      </c>
+      <c r="G29" t="s">
+        <v>16</v>
+      </c>
+      <c r="H29">
+        <v>2026</v>
+      </c>
+      <c r="I29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30">
         <v>2025</v>
       </c>
-      <c r="E29" t="s">
-        <v>52</v>
-      </c>
-      <c r="H29">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B30" t="s">
-        <v>81</v>
-      </c>
-      <c r="C30" t="s">
-        <v>82</v>
-      </c>
-      <c r="D30">
-        <v>2026</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
+        <v>13</v>
+      </c>
+      <c r="H30">
+        <v>2026</v>
+      </c>
+      <c r="I30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" t="s">
+        <v>146</v>
+      </c>
+      <c r="C31" t="s">
+        <v>147</v>
+      </c>
+      <c r="D31">
+        <v>2025</v>
+      </c>
+      <c r="G31" t="s">
+        <v>56</v>
+      </c>
+      <c r="H31">
+        <v>2026</v>
+      </c>
+      <c r="I31">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" t="s">
+        <v>22</v>
+      </c>
+      <c r="D32">
+        <v>2023</v>
+      </c>
+      <c r="E32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H32">
+        <v>2027</v>
+      </c>
+      <c r="I32">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" t="s">
+        <v>115</v>
+      </c>
+      <c r="C33" t="s">
+        <v>116</v>
+      </c>
+      <c r="D33">
+        <v>2026</v>
+      </c>
+      <c r="G33" t="s">
+        <v>40</v>
+      </c>
+      <c r="H33">
+        <v>2027</v>
+      </c>
+      <c r="I33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" t="s">
+        <v>117</v>
+      </c>
+      <c r="C34" t="s">
+        <v>118</v>
+      </c>
+      <c r="D34">
+        <v>2026</v>
+      </c>
+      <c r="F34" t="s">
         <v>38</v>
       </c>
-      <c r="H30">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>14</v>
-      </c>
-      <c r="B31" t="s">
-        <v>85</v>
-      </c>
-      <c r="C31" t="s">
-        <v>86</v>
-      </c>
-      <c r="D31">
-        <v>2026</v>
-      </c>
-      <c r="F31" t="s">
-        <v>33</v>
-      </c>
-      <c r="H31">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>14</v>
-      </c>
-      <c r="B32" t="s">
-        <v>87</v>
-      </c>
-      <c r="C32" t="s">
-        <v>88</v>
-      </c>
-      <c r="D32">
-        <v>2026</v>
-      </c>
-      <c r="G32" t="s">
-        <v>56</v>
-      </c>
-      <c r="H32">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B33" t="s">
-        <v>89</v>
-      </c>
-      <c r="C33" t="s">
-        <v>90</v>
-      </c>
-      <c r="D33">
-        <v>2026</v>
-      </c>
-      <c r="G33" t="s">
-        <v>19</v>
-      </c>
-      <c r="H33">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>14</v>
-      </c>
-      <c r="B34" t="s">
-        <v>91</v>
-      </c>
-      <c r="C34" t="s">
-        <v>92</v>
-      </c>
-      <c r="D34">
-        <v>2026</v>
-      </c>
-      <c r="G34" t="s">
-        <v>72</v>
-      </c>
       <c r="H34">
         <v>2027</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="B35" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C35" t="s">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="D35">
-        <v>2026</v>
-      </c>
-      <c r="G35" t="s">
-        <v>22</v>
+        <v>2025</v>
+      </c>
+      <c r="E35" t="s">
+        <v>10</v>
       </c>
       <c r="H35">
         <v>2027</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>14</v>
       </c>
       <c r="B36" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C36" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="D36">
         <v>2026</v>
       </c>
-      <c r="G36" t="s">
-        <v>47</v>
+      <c r="E36" t="s">
+        <v>107</v>
       </c>
       <c r="H36">
         <v>2027</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>14</v>
       </c>
       <c r="B37" t="s">
-        <v>96</v>
+        <v>29</v>
       </c>
       <c r="C37" t="s">
-        <v>97</v>
+        <v>30</v>
       </c>
       <c r="D37">
-        <v>2026</v>
-      </c>
-      <c r="G37" t="s">
-        <v>98</v>
+        <v>2024</v>
+      </c>
+      <c r="E37" t="s">
+        <v>31</v>
       </c>
       <c r="H37">
         <v>2027</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>14</v>
       </c>
       <c r="B38" t="s">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="C38" t="s">
-        <v>100</v>
+        <v>51</v>
       </c>
       <c r="D38">
-        <v>2026</v>
-      </c>
-      <c r="G38" t="s">
-        <v>101</v>
+        <v>2025</v>
+      </c>
+      <c r="E38" t="s">
+        <v>52</v>
       </c>
       <c r="H38">
         <v>2027</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B39" t="s">
-        <v>102</v>
+        <v>130</v>
       </c>
       <c r="C39" t="s">
-        <v>103</v>
+        <v>131</v>
       </c>
       <c r="D39">
         <v>2026</v>
       </c>
       <c r="G39" t="s">
-        <v>104</v>
+        <v>132</v>
       </c>
       <c r="H39">
         <v>2027</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I39">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="B40" t="s">
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="C40" t="s">
-        <v>106</v>
+        <v>47</v>
       </c>
       <c r="D40">
         <v>2026</v>
       </c>
       <c r="E40" t="s">
-        <v>107</v>
+        <v>38</v>
+      </c>
+      <c r="G40" t="s">
+        <v>47</v>
       </c>
       <c r="H40">
         <v>2027</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I40">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="B41" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="C41" t="s">
-        <v>158</v>
+        <v>138</v>
       </c>
       <c r="D41">
         <v>2026</v>
       </c>
-      <c r="E41" t="s">
-        <v>52</v>
+      <c r="G41" t="s">
+        <v>47</v>
       </c>
       <c r="H41">
         <v>2027</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I41">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="C42" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="D42">
         <v>2026</v>
       </c>
-      <c r="E42" t="s">
-        <v>107</v>
+      <c r="F42" t="s">
+        <v>38</v>
       </c>
       <c r="H42">
         <v>2027</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I42">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
-        <v>154</v>
+        <v>108</v>
       </c>
       <c r="C43" t="s">
-        <v>156</v>
+        <v>109</v>
       </c>
       <c r="D43">
         <v>2026</v>
       </c>
-      <c r="E43" t="s">
-        <v>31</v>
+      <c r="F43" t="s">
+        <v>38</v>
       </c>
       <c r="H43">
         <v>2027</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="B44" t="s">
-        <v>70</v>
+        <v>136</v>
       </c>
       <c r="C44" t="s">
-        <v>44</v>
+        <v>135</v>
       </c>
       <c r="D44">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E44" t="s">
         <v>10</v>
       </c>
       <c r="H44">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2028</v>
+      </c>
+      <c r="I44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>42</v>
       </c>
       <c r="B45" t="s">
-        <v>141</v>
+        <v>43</v>
       </c>
       <c r="C45" t="s">
-        <v>142</v>
+        <v>44</v>
       </c>
       <c r="D45">
-        <v>2026</v>
-      </c>
-      <c r="G45" t="s">
-        <v>22</v>
+        <v>2024</v>
+      </c>
+      <c r="E45" t="s">
+        <v>10</v>
       </c>
       <c r="H45">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2028</v>
+      </c>
+      <c r="I45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="C46" t="s">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="D46">
-        <v>2016</v>
+        <v>2024</v>
       </c>
       <c r="E46" t="s">
         <v>10</v>
       </c>
       <c r="H46">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2028</v>
+      </c>
+      <c r="I46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>122</v>
+      </c>
+      <c r="B47" t="s">
+        <v>171</v>
+      </c>
+      <c r="C47" t="s">
+        <v>40</v>
+      </c>
+      <c r="D47">
+        <v>2024</v>
+      </c>
+      <c r="E47" t="s">
+        <v>10</v>
+      </c>
+      <c r="H47">
+        <v>2028</v>
+      </c>
+      <c r="I47">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>17</v>
+      </c>
+      <c r="B48" t="s">
+        <v>39</v>
+      </c>
+      <c r="C48" t="s">
+        <v>40</v>
+      </c>
+      <c r="D48">
+        <v>2024</v>
+      </c>
+      <c r="E48" t="s">
+        <v>10</v>
+      </c>
+      <c r="H48">
+        <v>2028</v>
+      </c>
+      <c r="I48">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>59</v>
+      </c>
+      <c r="B49" t="s">
+        <v>125</v>
+      </c>
+      <c r="C49" t="s">
+        <v>126</v>
+      </c>
+      <c r="D49">
+        <v>2026</v>
+      </c>
+      <c r="E49" t="s">
+        <v>10</v>
+      </c>
+      <c r="H49">
+        <v>2029</v>
+      </c>
+      <c r="I49">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>14</v>
+      </c>
+      <c r="B50" t="s">
+        <v>83</v>
+      </c>
+      <c r="C50" t="s">
+        <v>84</v>
+      </c>
+      <c r="D50">
+        <v>2025</v>
+      </c>
+      <c r="F50" t="s">
+        <v>10</v>
+      </c>
+      <c r="H50">
+        <v>2029</v>
+      </c>
+      <c r="I50">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>17</v>
+      </c>
+      <c r="B51" t="s">
+        <v>55</v>
+      </c>
+      <c r="C51" t="s">
+        <v>56</v>
+      </c>
+      <c r="D51">
+        <v>2025</v>
+      </c>
+      <c r="E51" t="s">
+        <v>38</v>
+      </c>
+      <c r="H51">
+        <v>2029</v>
+      </c>
+      <c r="I51">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>7</v>
       </c>
-      <c r="B47" t="s">
-        <v>127</v>
-      </c>
-      <c r="C47" t="s">
-        <v>128</v>
-      </c>
-      <c r="D47">
-        <v>2026</v>
-      </c>
-      <c r="G47" t="s">
+      <c r="B52" t="s">
+        <v>129</v>
+      </c>
+      <c r="C52" t="s">
         <v>40</v>
       </c>
-      <c r="H47">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>7</v>
-      </c>
-      <c r="B48" t="s">
-        <v>130</v>
-      </c>
-      <c r="C48" t="s">
-        <v>131</v>
-      </c>
-      <c r="D48">
-        <v>2026</v>
-      </c>
-      <c r="G48" t="s">
-        <v>132</v>
-      </c>
-      <c r="H48">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>7</v>
-      </c>
-      <c r="B49" t="s">
-        <v>148</v>
-      </c>
-      <c r="C49" t="s">
-        <v>150</v>
-      </c>
-      <c r="D49">
-        <v>2026</v>
-      </c>
-      <c r="G49" t="s">
+      <c r="D52">
+        <v>2026</v>
+      </c>
+      <c r="E52" t="s">
+        <v>10</v>
+      </c>
+      <c r="H52">
+        <v>2030</v>
+      </c>
+      <c r="I52">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>59</v>
+      </c>
+      <c r="B53" t="s">
+        <v>149</v>
+      </c>
+      <c r="C53" t="s">
+        <v>151</v>
+      </c>
+      <c r="D53">
+        <v>2025</v>
+      </c>
+      <c r="G53" t="s">
         <v>40</v>
       </c>
-      <c r="H49">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>26</v>
-      </c>
-      <c r="B50" t="s">
-        <v>27</v>
-      </c>
-      <c r="C50" t="s">
-        <v>28</v>
-      </c>
-      <c r="D50">
-        <v>2023</v>
-      </c>
-      <c r="E50" t="s">
-        <v>10</v>
-      </c>
-      <c r="H50">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>26</v>
-      </c>
-      <c r="B51" t="s">
-        <v>137</v>
-      </c>
-      <c r="C51" t="s">
-        <v>138</v>
-      </c>
-      <c r="D51">
-        <v>2026</v>
-      </c>
-      <c r="G51" t="s">
-        <v>47</v>
-      </c>
-      <c r="H51">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>26</v>
-      </c>
-      <c r="B52" t="s">
-        <v>139</v>
-      </c>
-      <c r="C52" t="s">
-        <v>140</v>
-      </c>
-      <c r="D52">
-        <v>2026</v>
-      </c>
-      <c r="F52" t="s">
-        <v>38</v>
-      </c>
-      <c r="H52">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>26</v>
-      </c>
-      <c r="B53" t="s">
-        <v>145</v>
-      </c>
-      <c r="C53" t="s">
-        <v>47</v>
-      </c>
-      <c r="D53">
-        <v>2026</v>
-      </c>
-      <c r="E53" t="s">
-        <v>38</v>
-      </c>
-      <c r="G53" t="s">
-        <v>47</v>
-      </c>
       <c r="H53">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2026</v>
+      </c>
+      <c r="I53">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="B54" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C54" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="D54">
         <v>2025</v>
       </c>
-      <c r="E54" t="s">
+      <c r="G54" t="s">
+        <v>9</v>
+      </c>
+      <c r="H54">
+        <v>2026</v>
+      </c>
+      <c r="I54">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>14</v>
+      </c>
+      <c r="B55" t="s">
+        <v>48</v>
+      </c>
+      <c r="C55" t="s">
+        <v>49</v>
+      </c>
+      <c r="D55">
+        <v>2025</v>
+      </c>
+      <c r="G55" t="s">
+        <v>40</v>
+      </c>
+      <c r="H55">
+        <v>2026</v>
+      </c>
+      <c r="I55">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>11</v>
+      </c>
+      <c r="B56" t="s">
+        <v>12</v>
+      </c>
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56">
+        <v>2021</v>
+      </c>
+      <c r="E56" t="s">
         <v>10</v>
       </c>
-      <c r="H54">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>45</v>
-      </c>
-      <c r="B55" t="s">
-        <v>143</v>
-      </c>
-      <c r="C55" t="s">
-        <v>144</v>
-      </c>
-      <c r="D55">
-        <v>2026</v>
-      </c>
-      <c r="G55" t="s">
-        <v>72</v>
-      </c>
-      <c r="H55">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+      <c r="H56">
+        <v>2026</v>
+      </c>
+      <c r="I56">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>122</v>
       </c>
-      <c r="B56" t="s">
-        <v>123</v>
-      </c>
-      <c r="C56" t="s">
-        <v>124</v>
-      </c>
-      <c r="D56">
-        <v>2026</v>
-      </c>
-      <c r="G56" t="s">
+      <c r="B57" t="s">
+        <v>57</v>
+      </c>
+      <c r="C57" t="s">
+        <v>58</v>
+      </c>
+      <c r="D57">
+        <v>2025</v>
+      </c>
+      <c r="G57" t="s">
         <v>40</v>
       </c>
-      <c r="H56">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>17</v>
-      </c>
-      <c r="B57" t="s">
-        <v>18</v>
-      </c>
-      <c r="C57" t="s">
-        <v>19</v>
-      </c>
-      <c r="D57">
-        <v>2023</v>
-      </c>
-      <c r="E57" t="s">
-        <v>10</v>
-      </c>
       <c r="H57">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2026</v>
+      </c>
+      <c r="I57">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>17</v>
       </c>
       <c r="B58" t="s">
-        <v>108</v>
+        <v>53</v>
       </c>
       <c r="C58" t="s">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="D58">
-        <v>2026</v>
-      </c>
-      <c r="F58" t="s">
-        <v>38</v>
+        <v>2025</v>
+      </c>
+      <c r="G58" t="s">
+        <v>40</v>
       </c>
       <c r="H58">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2026</v>
+      </c>
+      <c r="I58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B59" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="C59" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="D59">
         <v>2026</v>
       </c>
       <c r="G59" t="s">
-        <v>56</v>
+        <v>121</v>
       </c>
       <c r="H59">
         <v>2027</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I59">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B60" t="s">
-        <v>112</v>
+        <v>153</v>
       </c>
       <c r="C60" t="s">
-        <v>109</v>
+        <v>157</v>
       </c>
       <c r="D60">
         <v>2026</v>
       </c>
-      <c r="G60" t="s">
-        <v>19</v>
+      <c r="E60" t="s">
+        <v>107</v>
       </c>
       <c r="H60">
         <v>2027</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I60">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B61" t="s">
-        <v>41</v>
+        <v>154</v>
       </c>
       <c r="C61" t="s">
-        <v>40</v>
+        <v>156</v>
       </c>
       <c r="D61">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="E61" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="H61">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I61">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B62" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="C62" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="D62">
         <v>2026</v>
       </c>
       <c r="E62" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="H62">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I62">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>14</v>
       </c>
       <c r="B63" t="s">
-        <v>32</v>
+        <v>96</v>
       </c>
       <c r="C63" t="s">
-        <v>16</v>
+        <v>97</v>
       </c>
       <c r="D63">
-        <v>2024</v>
-      </c>
-      <c r="E63" t="s">
-        <v>33</v>
+        <v>2026</v>
+      </c>
+      <c r="G63" t="s">
+        <v>98</v>
       </c>
       <c r="H63">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I63">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>14</v>
       </c>
       <c r="B64" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="C64" t="s">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="D64">
-        <v>2024</v>
-      </c>
-      <c r="E64" t="s">
-        <v>36</v>
+        <v>2026</v>
+      </c>
+      <c r="G64" t="s">
+        <v>101</v>
       </c>
       <c r="H64">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I64">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>14</v>
       </c>
       <c r="B65" t="s">
-        <v>37</v>
+        <v>102</v>
       </c>
       <c r="C65" t="s">
-        <v>19</v>
+        <v>103</v>
       </c>
       <c r="D65">
-        <v>2024</v>
-      </c>
-      <c r="E65" t="s">
-        <v>38</v>
+        <v>2026</v>
+      </c>
+      <c r="G65" t="s">
+        <v>104</v>
       </c>
       <c r="H65">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I65">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>42</v>
       </c>
       <c r="B66" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="C66" t="s">
         <v>44</v>
       </c>
       <c r="D66">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E66" t="s">
         <v>10</v>
       </c>
       <c r="H66">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I66">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>169</v>
+        <v>42</v>
       </c>
       <c r="B67" t="s">
-        <v>168</v>
+        <v>141</v>
       </c>
       <c r="C67" t="s">
-        <v>40</v>
+        <v>142</v>
       </c>
       <c r="D67">
-        <v>2024</v>
-      </c>
-      <c r="E67" t="s">
-        <v>10</v>
+        <v>2026</v>
+      </c>
+      <c r="G67" t="s">
+        <v>22</v>
       </c>
       <c r="H67">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I67">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="B68" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C68" t="s">
-        <v>47</v>
+        <v>9</v>
       </c>
       <c r="D68">
-        <v>2024</v>
+        <v>2016</v>
       </c>
       <c r="E68" t="s">
         <v>10</v>
       </c>
       <c r="H68">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I68">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>122</v>
+        <v>7</v>
       </c>
       <c r="B69" t="s">
-        <v>171</v>
+        <v>148</v>
       </c>
       <c r="C69" t="s">
+        <v>150</v>
+      </c>
+      <c r="D69">
+        <v>2026</v>
+      </c>
+      <c r="G69" t="s">
         <v>40</v>
       </c>
-      <c r="D69">
-        <v>2024</v>
-      </c>
-      <c r="E69" t="s">
-        <v>10</v>
-      </c>
       <c r="H69">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I69">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B70" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="C70" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="D70">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E70" t="s">
         <v>10</v>
       </c>
       <c r="H70">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I70">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="B71" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="C71" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="D71">
         <v>2026</v>
       </c>
-      <c r="E71" t="s">
-        <v>10</v>
+      <c r="G71" t="s">
+        <v>72</v>
       </c>
       <c r="H71">
-        <v>2029</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I71">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>14</v>
+        <v>122</v>
       </c>
       <c r="B72" t="s">
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="C72" t="s">
-        <v>84</v>
+        <v>124</v>
       </c>
       <c r="D72">
-        <v>2025</v>
-      </c>
-      <c r="F72" t="s">
-        <v>10</v>
+        <v>2026</v>
+      </c>
+      <c r="G72" t="s">
+        <v>40</v>
       </c>
       <c r="H72">
-        <v>2029</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I72">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>17</v>
       </c>
       <c r="B73" t="s">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="C73" t="s">
+        <v>111</v>
+      </c>
+      <c r="D73">
+        <v>2026</v>
+      </c>
+      <c r="G73" t="s">
         <v>56</v>
       </c>
-      <c r="D73">
-        <v>2025</v>
-      </c>
-      <c r="E73" t="s">
-        <v>38</v>
-      </c>
       <c r="H73">
-        <v>2029</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I73">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B74" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="C74" t="s">
-        <v>40</v>
+        <v>109</v>
       </c>
       <c r="D74">
         <v>2026</v>
       </c>
-      <c r="E74" t="s">
-        <v>10</v>
+      <c r="G74" t="s">
+        <v>19</v>
       </c>
       <c r="H74">
-        <v>2030</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2027</v>
+      </c>
+      <c r="I74">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>169</v>
+        <v>14</v>
       </c>
       <c r="B75" t="s">
-        <v>167</v>
+        <v>34</v>
       </c>
       <c r="C75" t="s">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="D75">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="E75" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="H75">
-        <v>2030</v>
+        <v>2028</v>
+      </c>
+      <c r="I75">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H75">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I75">
+    <sortCondition ref="I2:I75"/>
     <sortCondition ref="H2:H75"/>
     <sortCondition ref="A2:A75"/>
   </sortState>

</xml_diff>

<commit_message>
Add International Football greatest games, women's rivalries, and fix NBA arena naming. Women's College Basketball and NWSL/WSL/Liga F clubs gain the Rivalries row and the /sports/rivalries board. New International Football greatest games: a top-50 board with a decade filter on the national hub, a top-10 list on every national team page, and the section leads the cross-sport Greatest Games page ahead of the NFL, with the 1954, 1966 and 2022 finals carrying video; men's tournament matches only, 2026 World Cup held until the tournament ends. NBA top games now show the arena name as of the game (Delta Center, not Vivint Arena) on the hub, the Greatest Games page and team pages by carrying arena_as_of on the league-wide rows and preferring it over the canonical name.
</commit_message>
<xml_diff>
--- a/ZoneZero_Champions.xlsx
+++ b/ZoneZero_Champions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashwi\Desktop\Projects\Metro Area Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5A6CCF-8B08-46A7-BA11-5AE1A9590AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62530FD4-2FE1-4D6D-AD11-7BEC9C33100E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="360" windowWidth="36675" windowHeight="16725" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="480" windowWidth="24600" windowHeight="16650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,31 +41,7 @@
     <author>Ashwin Desikan</author>
   </authors>
   <commentList>
-    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{AB9676B4-875A-49BB-B97A-23D16A7B1B08}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Ashwin Desikan:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-2025 Men's College World Series finals Game 2, LSU bt Coastal Carolina 5-3. Source: NCAA.com, https://www.ncaa.com/live-updates/baseball/d1/lsu-wins-2025-mens-college-world-series</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D4" authorId="0" shapeId="0" xr:uid="{7288B152-5BC5-46F2-929C-3CC1643389D0}">
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{7288B152-5BC5-46F2-929C-3CC1643389D0}">
       <text>
         <r>
           <rPr>
@@ -89,7 +65,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D9" authorId="0" shapeId="0" xr:uid="{BAC8AF97-7BA7-4D30-9D9B-CB56DEF85C32}">
+    <comment ref="D7" authorId="0" shapeId="0" xr:uid="{BAC8AF97-7BA7-4D30-9D9B-CB56DEF85C32}">
       <text>
         <r>
           <rPr>
@@ -113,7 +89,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D12" authorId="0" shapeId="0" xr:uid="{C39B794B-050A-4081-ABC9-A3B1650982CF}">
+    <comment ref="D10" authorId="0" shapeId="0" xr:uid="{C39B794B-050A-4081-ABC9-A3B1650982CF}">
       <text>
         <r>
           <rPr>
@@ -137,7 +113,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{B7459AF6-2CBF-4B87-AB77-A1AD1DADDD58}">
+    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{B7459AF6-2CBF-4B87-AB77-A1AD1DADDD58}">
       <text>
         <r>
           <rPr>
@@ -161,7 +137,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D14" authorId="0" shapeId="0" xr:uid="{D0765079-216E-4F66-9BD0-BE443833BDFA}">
+    <comment ref="D12" authorId="0" shapeId="0" xr:uid="{D0765079-216E-4F66-9BD0-BE443833BDFA}">
       <text>
         <r>
           <rPr>
@@ -185,7 +161,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D15" authorId="0" shapeId="0" xr:uid="{EEFFDEB6-2AA9-4E65-802E-B73E90A8FBA3}">
+    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{EEFFDEB6-2AA9-4E65-802E-B73E90A8FBA3}">
       <text>
         <r>
           <rPr>
@@ -209,7 +185,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D16" authorId="0" shapeId="0" xr:uid="{3FBB27D6-DAAA-4FA7-B404-53035B7FC7A0}">
+    <comment ref="D14" authorId="0" shapeId="0" xr:uid="{3FBB27D6-DAAA-4FA7-B404-53035B7FC7A0}">
       <text>
         <r>
           <rPr>
@@ -233,7 +209,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D17" authorId="0" shapeId="0" xr:uid="{314A5A24-E37B-4766-B160-7A6A96BB8442}">
+    <comment ref="D15" authorId="0" shapeId="0" xr:uid="{314A5A24-E37B-4766-B160-7A6A96BB8442}">
       <text>
         <r>
           <rPr>
@@ -257,7 +233,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{5A41BE4B-4C4F-4605-A4E5-38E8AA2631E5}">
+    <comment ref="D16" authorId="0" shapeId="0" xr:uid="{5A41BE4B-4C4F-4605-A4E5-38E8AA2631E5}">
       <text>
         <r>
           <rPr>
@@ -281,7 +257,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D19" authorId="0" shapeId="0" xr:uid="{2E01140C-023C-40EE-AD29-5767C5D25E2A}">
+    <comment ref="D17" authorId="0" shapeId="0" xr:uid="{2E01140C-023C-40EE-AD29-5767C5D25E2A}">
       <text>
         <r>
           <rPr>
@@ -305,7 +281,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D20" authorId="0" shapeId="0" xr:uid="{A812C2D5-8246-4A5F-B8F3-009F3F8C1EA9}">
+    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{A812C2D5-8246-4A5F-B8F3-009F3F8C1EA9}">
       <text>
         <r>
           <rPr>
@@ -329,7 +305,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{34CC526B-6E4B-4BBD-9150-0FD093A82256}">
+    <comment ref="D19" authorId="0" shapeId="0" xr:uid="{34CC526B-6E4B-4BBD-9150-0FD093A82256}">
       <text>
         <r>
           <rPr>
@@ -353,7 +329,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{8F508446-BE66-464F-A9EB-76AF07BF3424}">
+    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{8F508446-BE66-464F-A9EB-76AF07BF3424}">
       <text>
         <r>
           <rPr>
@@ -377,7 +353,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D24" authorId="0" shapeId="0" xr:uid="{6834CD08-48FC-4182-BBA5-801595B4D4F0}">
+    <comment ref="D22" authorId="0" shapeId="0" xr:uid="{6834CD08-48FC-4182-BBA5-801595B4D4F0}">
       <text>
         <r>
           <rPr>
@@ -401,7 +377,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D25" authorId="0" shapeId="0" xr:uid="{329433DE-BFFB-49F7-AFAE-4261991DD1B2}">
+    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{329433DE-BFFB-49F7-AFAE-4261991DD1B2}">
       <text>
         <r>
           <rPr>
@@ -425,7 +401,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D26" authorId="0" shapeId="0" xr:uid="{41F91886-A3B1-437C-AEE3-46C58843CC08}">
+    <comment ref="D24" authorId="0" shapeId="0" xr:uid="{41F91886-A3B1-437C-AEE3-46C58843CC08}">
       <text>
         <r>
           <rPr>
@@ -449,7 +425,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D29" authorId="0" shapeId="0" xr:uid="{DF158B7E-72F4-44BF-AA37-16502ADB7DB7}">
+    <comment ref="D27" authorId="0" shapeId="0" xr:uid="{DF158B7E-72F4-44BF-AA37-16502ADB7DB7}">
       <text>
         <r>
           <rPr>
@@ -473,7 +449,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D31" authorId="0" shapeId="0" xr:uid="{42F0BA49-73AA-40F5-AEEE-90BB9EB3DF02}">
+    <comment ref="D29" authorId="0" shapeId="0" xr:uid="{42F0BA49-73AA-40F5-AEEE-90BB9EB3DF02}">
       <text>
         <r>
           <rPr>
@@ -497,7 +473,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D32" authorId="0" shapeId="0" xr:uid="{784244AE-2833-41B4-BBA5-15801F62CC0A}">
+    <comment ref="D30" authorId="0" shapeId="0" xr:uid="{784244AE-2833-41B4-BBA5-15801F62CC0A}">
       <text>
         <r>
           <rPr>
@@ -521,7 +497,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D34" authorId="0" shapeId="0" xr:uid="{E7DC1F20-4411-45EE-9207-6EA393E2DA86}">
+    <comment ref="D32" authorId="0" shapeId="0" xr:uid="{E7DC1F20-4411-45EE-9207-6EA393E2DA86}">
       <text>
         <r>
           <rPr>
@@ -545,7 +521,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D35" authorId="0" shapeId="0" xr:uid="{38ADAA7A-DA34-4DD7-9B66-AA8EBEBFDC69}">
+    <comment ref="D33" authorId="0" shapeId="0" xr:uid="{38ADAA7A-DA34-4DD7-9B66-AA8EBEBFDC69}">
       <text>
         <r>
           <rPr>
@@ -569,7 +545,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D36" authorId="0" shapeId="0" xr:uid="{D637E791-FC2B-4471-932F-5BD32D56F951}">
+    <comment ref="D34" authorId="0" shapeId="0" xr:uid="{D637E791-FC2B-4471-932F-5BD32D56F951}">
       <text>
         <r>
           <rPr>
@@ -583,7 +559,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D37" authorId="0" shapeId="0" xr:uid="{518AD3BD-73B5-45D8-8D44-ABEE10E52FD7}">
+    <comment ref="D35" authorId="0" shapeId="0" xr:uid="{518AD3BD-73B5-45D8-8D44-ABEE10E52FD7}">
       <text>
         <r>
           <rPr>
@@ -607,7 +583,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D38" authorId="0" shapeId="0" xr:uid="{37AA12B4-FF62-4659-B1BB-EE0BAACD0AA6}">
+    <comment ref="D36" authorId="0" shapeId="0" xr:uid="{37AA12B4-FF62-4659-B1BB-EE0BAACD0AA6}">
       <text>
         <r>
           <rPr>
@@ -631,7 +607,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D39" authorId="0" shapeId="0" xr:uid="{407D07C7-1E5A-4174-B8EE-A048BA11CF08}">
+    <comment ref="D37" authorId="0" shapeId="0" xr:uid="{407D07C7-1E5A-4174-B8EE-A048BA11CF08}">
       <text>
         <r>
           <rPr>
@@ -655,7 +631,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D40" authorId="0" shapeId="0" xr:uid="{54AE28CE-8BC2-4F7B-B2A3-C9D6038D253D}">
+    <comment ref="D38" authorId="0" shapeId="0" xr:uid="{54AE28CE-8BC2-4F7B-B2A3-C9D6038D253D}">
       <text>
         <r>
           <rPr>
@@ -679,7 +655,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{7646D5E9-7FB5-4350-BF05-5F23EDA92E86}">
+    <comment ref="D39" authorId="0" shapeId="0" xr:uid="{7646D5E9-7FB5-4350-BF05-5F23EDA92E86}">
       <text>
         <r>
           <rPr>
@@ -693,7 +669,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D43" authorId="0" shapeId="0" xr:uid="{FEB59916-5634-41AE-A104-DE61E763A409}">
+    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{FEB59916-5634-41AE-A104-DE61E763A409}">
       <text>
         <r>
           <rPr>
@@ -717,7 +693,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D44" authorId="0" shapeId="0" xr:uid="{2E199270-073E-4D7F-AB36-33BA722B4E37}">
+    <comment ref="D42" authorId="0" shapeId="0" xr:uid="{2E199270-073E-4D7F-AB36-33BA722B4E37}">
       <text>
         <r>
           <rPr>
@@ -741,7 +717,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D45" authorId="0" shapeId="0" xr:uid="{DFD5A8E1-FA58-4A5D-9FD6-7C82E172B5B2}">
+    <comment ref="D43" authorId="0" shapeId="0" xr:uid="{DFD5A8E1-FA58-4A5D-9FD6-7C82E172B5B2}">
       <text>
         <r>
           <rPr>
@@ -765,7 +741,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D46" authorId="0" shapeId="0" xr:uid="{AFE554BD-C0D8-48CB-868B-082F4AFB5BF4}">
+    <comment ref="D44" authorId="0" shapeId="0" xr:uid="{AFE554BD-C0D8-48CB-868B-082F4AFB5BF4}">
       <text>
         <r>
           <rPr>
@@ -789,7 +765,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D47" authorId="0" shapeId="0" xr:uid="{8D255B0D-EC77-4323-AA63-A1BBBDD4AEA3}">
+    <comment ref="D45" authorId="0" shapeId="0" xr:uid="{8D255B0D-EC77-4323-AA63-A1BBBDD4AEA3}">
       <text>
         <r>
           <rPr>
@@ -803,7 +779,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D48" authorId="0" shapeId="0" xr:uid="{1DFEB1AC-A641-436D-B8B0-9E15A4D19BF2}">
+    <comment ref="D46" authorId="0" shapeId="0" xr:uid="{1DFEB1AC-A641-436D-B8B0-9E15A4D19BF2}">
       <text>
         <r>
           <rPr>
@@ -817,7 +793,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D49" authorId="0" shapeId="0" xr:uid="{6F4D585C-957F-4F2D-9534-B216BF0CEF98}">
+    <comment ref="D47" authorId="0" shapeId="0" xr:uid="{6F4D585C-957F-4F2D-9534-B216BF0CEF98}">
       <text>
         <r>
           <rPr>
@@ -841,7 +817,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D50" authorId="0" shapeId="0" xr:uid="{719A10D4-C6B0-4B96-A328-8054C69D372B}">
+    <comment ref="D48" authorId="0" shapeId="0" xr:uid="{719A10D4-C6B0-4B96-A328-8054C69D372B}">
       <text>
         <r>
           <rPr>
@@ -865,7 +841,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{6F1B4FBE-65F9-4E7C-80B1-05C8D4DAE7CC}">
+    <comment ref="D49" authorId="0" shapeId="0" xr:uid="{6F1B4FBE-65F9-4E7C-80B1-05C8D4DAE7CC}">
       <text>
         <r>
           <rPr>
@@ -889,7 +865,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D52" authorId="0" shapeId="0" xr:uid="{A47217EE-9271-43EB-90FE-8F83610DA1D4}">
+    <comment ref="D50" authorId="0" shapeId="0" xr:uid="{A47217EE-9271-43EB-90FE-8F83610DA1D4}">
       <text>
         <r>
           <rPr>
@@ -913,7 +889,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D53" authorId="0" shapeId="0" xr:uid="{533FF206-6AA1-4BFA-BC92-9D8B3064C39D}">
+    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{533FF206-6AA1-4BFA-BC92-9D8B3064C39D}">
       <text>
         <r>
           <rPr>
@@ -937,7 +913,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D54" authorId="0" shapeId="0" xr:uid="{2066D358-FE86-4958-A4DB-5940778115D3}">
+    <comment ref="D52" authorId="0" shapeId="0" xr:uid="{2066D358-FE86-4958-A4DB-5940778115D3}">
       <text>
         <r>
           <rPr>
@@ -961,7 +937,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D55" authorId="0" shapeId="0" xr:uid="{2A752479-3D04-461B-983A-820DC3216B4E}">
+    <comment ref="D53" authorId="0" shapeId="0" xr:uid="{2A752479-3D04-461B-983A-820DC3216B4E}">
       <text>
         <r>
           <rPr>
@@ -985,7 +961,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D56" authorId="0" shapeId="0" xr:uid="{B552DA13-90D7-4D7A-868B-DC7BEEA87181}">
+    <comment ref="D54" authorId="0" shapeId="0" xr:uid="{B552DA13-90D7-4D7A-868B-DC7BEEA87181}">
       <text>
         <r>
           <rPr>
@@ -1009,7 +985,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D58" authorId="0" shapeId="0" xr:uid="{A05DF8EC-83C9-4620-9EDE-0D5A094D59EB}">
+    <comment ref="D56" authorId="0" shapeId="0" xr:uid="{A05DF8EC-83C9-4620-9EDE-0D5A094D59EB}">
       <text>
         <r>
           <rPr>
@@ -1033,7 +1009,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D59" authorId="0" shapeId="0" xr:uid="{0A00B11F-49D6-46F1-9DA8-5EF8D1F5EEC7}">
+    <comment ref="D57" authorId="0" shapeId="0" xr:uid="{0A00B11F-49D6-46F1-9DA8-5EF8D1F5EEC7}">
       <text>
         <r>
           <rPr>
@@ -1057,7 +1033,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D61" authorId="0" shapeId="0" xr:uid="{6EF7E574-83D5-4512-814C-4EAA7D554E0F}">
+    <comment ref="D59" authorId="0" shapeId="0" xr:uid="{6EF7E574-83D5-4512-814C-4EAA7D554E0F}">
       <text>
         <r>
           <rPr>
@@ -1081,7 +1057,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D62" authorId="0" shapeId="0" xr:uid="{BA4BFA91-5E1E-4F4E-B781-56CE4914BA5A}">
+    <comment ref="D60" authorId="0" shapeId="0" xr:uid="{BA4BFA91-5E1E-4F4E-B781-56CE4914BA5A}">
       <text>
         <r>
           <rPr>
@@ -1105,7 +1081,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D63" authorId="0" shapeId="0" xr:uid="{54B4E860-83AD-4400-93D7-E31540965980}">
+    <comment ref="D61" authorId="0" shapeId="0" xr:uid="{54B4E860-83AD-4400-93D7-E31540965980}">
       <text>
         <r>
           <rPr>
@@ -1129,7 +1105,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D64" authorId="0" shapeId="0" xr:uid="{FEE7D06D-A1A8-43C9-97FC-71E9186F8D7D}">
+    <comment ref="D62" authorId="0" shapeId="0" xr:uid="{FEE7D06D-A1A8-43C9-97FC-71E9186F8D7D}">
       <text>
         <r>
           <rPr>
@@ -1398,7 +1374,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="201">
   <si>
     <t>Sport</t>
   </si>
@@ -1844,9 +1820,6 @@
     <t>Denver</t>
   </si>
   <si>
-    <t>LSU</t>
-  </si>
-  <si>
     <t>CONCACAF Champions Cup</t>
   </si>
   <si>
@@ -1998,6 +1971,12 @@
   </si>
   <si>
     <t>Next Awarded Date</t>
+  </si>
+  <si>
+    <t>Wyndham Clark</t>
+  </si>
+  <si>
+    <t>Oklahoma</t>
   </si>
 </sst>
 </file>
@@ -2041,18 +2020,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -2068,13 +2041,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2091,10 +2061,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2445,7 +2411,7 @@
     <col min="4" max="4" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2460,7 +2426,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -2471,34 +2437,34 @@
       <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>199</v>
+      <c r="H1" t="s">
+        <v>198</v>
       </c>
       <c r="I1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C2" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="D2" s="2">
-        <v>45830</v>
+        <v>45836</v>
       </c>
       <c r="G2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H2" s="4">
-        <v>46194</v>
+        <v>46</v>
+      </c>
+      <c r="H2" s="2">
+        <v>46200</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -2506,178 +2472,180 @@
         <v>170</v>
       </c>
       <c r="B3" t="s">
-        <v>183</v>
-      </c>
-      <c r="C3" s="3"/>
+        <v>192</v>
+      </c>
+      <c r="C3" t="s">
+        <v>185</v>
+      </c>
       <c r="D3" s="2">
-        <v>45830</v>
+        <v>45850</v>
       </c>
       <c r="E3" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="4">
-        <v>46194</v>
+      <c r="H3" s="2">
+        <v>46214</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>170</v>
       </c>
       <c r="B4" t="s">
-        <v>135</v>
+        <v>189</v>
       </c>
       <c r="C4" t="s">
-        <v>136</v>
+        <v>184</v>
       </c>
       <c r="D4" s="2">
-        <v>45836</v>
-      </c>
-      <c r="G4" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" s="4">
-        <v>46200</v>
+        <v>45851</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="2">
+        <v>46215</v>
       </c>
       <c r="I4">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B5" t="s">
-        <v>193</v>
+        <v>172</v>
       </c>
       <c r="C5" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="D5" s="2">
-        <v>45850</v>
+        <v>45858</v>
       </c>
       <c r="E5" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="4">
-        <v>46214</v>
+      <c r="H5" s="2">
+        <v>46222</v>
       </c>
       <c r="I5">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>171</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>190</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>185</v>
+        <v>15</v>
       </c>
       <c r="D6" s="2">
-        <v>45851</v>
+        <v>44913</v>
       </c>
       <c r="E6" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="4">
-        <v>46215</v>
+      <c r="H6" s="2">
+        <v>46222</v>
       </c>
       <c r="I6">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>170</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
       <c r="C7" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="D7" s="2">
-        <v>45858</v>
+        <v>45759</v>
       </c>
       <c r="E7" t="s">
-        <v>9</v>
-      </c>
-      <c r="H7" s="4">
-        <v>46222</v>
+        <v>35</v>
+      </c>
+      <c r="H7" s="2">
+        <v>46256</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>170</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>193</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>183</v>
       </c>
       <c r="D8" s="2">
-        <v>44913</v>
+        <v>45906</v>
       </c>
       <c r="E8" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="4">
-        <v>46222</v>
+      <c r="H8" s="2">
+        <v>46270</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>170</v>
       </c>
       <c r="B9" t="s">
-        <v>152</v>
+        <v>190</v>
       </c>
       <c r="C9" t="s">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="D9" s="2">
-        <v>45759</v>
+        <v>45907</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
-      </c>
-      <c r="H9" s="4">
-        <v>46256</v>
+        <v>9</v>
+      </c>
+      <c r="H9" s="2">
+        <v>46271</v>
       </c>
       <c r="I9">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>171</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>194</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>184</v>
+        <v>67</v>
       </c>
       <c r="D10" s="2">
-        <v>45906</v>
-      </c>
-      <c r="E10" t="s">
-        <v>9</v>
-      </c>
-      <c r="H10" s="4">
-        <v>46270</v>
+        <v>45927</v>
+      </c>
+      <c r="G10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="2">
+        <v>46291</v>
       </c>
       <c r="I10">
         <v>2</v>
@@ -2685,68 +2653,68 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>171</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>191</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>181</v>
+        <v>64</v>
       </c>
       <c r="D11" s="2">
-        <v>45907</v>
-      </c>
-      <c r="E11" t="s">
-        <v>9</v>
-      </c>
-      <c r="H11" s="4">
-        <v>46271</v>
+        <v>45935</v>
+      </c>
+      <c r="G11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="2">
+        <v>46299</v>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="D12" s="2">
-        <v>45927</v>
+        <v>45940</v>
       </c>
       <c r="G12" t="s">
-        <v>12</v>
-      </c>
-      <c r="H12" s="4">
-        <v>46291</v>
+        <v>39</v>
+      </c>
+      <c r="H12" s="2">
+        <v>46304</v>
       </c>
       <c r="I12">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D13" s="2">
-        <v>45935</v>
+        <v>45960</v>
       </c>
       <c r="G13" t="s">
-        <v>12</v>
-      </c>
-      <c r="H13" s="4">
-        <v>46299</v>
+        <v>62</v>
+      </c>
+      <c r="H13" s="2">
+        <v>46324</v>
       </c>
       <c r="I13">
         <v>3</v>
@@ -2754,91 +2722,91 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>120</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
-        <v>56</v>
+        <v>194</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D14" s="2">
-        <v>45940</v>
+        <v>45962</v>
       </c>
       <c r="G14" t="s">
         <v>39</v>
       </c>
-      <c r="H14" s="4">
-        <v>46304</v>
+      <c r="H14" s="2">
+        <v>46326</v>
       </c>
       <c r="I14">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="D15" s="2">
-        <v>45960</v>
-      </c>
-      <c r="G15" t="s">
-        <v>62</v>
-      </c>
-      <c r="H15" s="4">
-        <v>46324</v>
+        <v>44884</v>
+      </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
+      <c r="H15" s="2">
+        <v>46333</v>
       </c>
       <c r="I15">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>195</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="D16" s="2">
-        <v>45962</v>
+        <v>45977</v>
       </c>
       <c r="G16" t="s">
-        <v>39</v>
-      </c>
-      <c r="H16" s="4">
-        <v>46326</v>
+        <v>8</v>
+      </c>
+      <c r="H16" s="2">
+        <v>46341</v>
       </c>
       <c r="I16">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="D17" s="2">
-        <v>44884</v>
-      </c>
-      <c r="E17" t="s">
-        <v>9</v>
-      </c>
-      <c r="H17" s="4">
-        <v>46333</v>
+        <v>45983</v>
+      </c>
+      <c r="G17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H17" s="2">
+        <v>46347</v>
       </c>
       <c r="I17">
         <v>4</v>
@@ -2846,71 +2814,71 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D18" s="2">
-        <v>45977</v>
-      </c>
-      <c r="G18" t="s">
-        <v>8</v>
-      </c>
-      <c r="H18" s="4">
-        <v>46341</v>
+        <v>45990</v>
+      </c>
+      <c r="F18" t="s">
+        <v>32</v>
+      </c>
+      <c r="H18" s="2">
+        <v>46354</v>
       </c>
       <c r="I18">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>158</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="D19" s="2">
-        <v>45983</v>
+        <v>45994</v>
       </c>
       <c r="G19" t="s">
-        <v>39</v>
-      </c>
-      <c r="H19" s="4">
-        <v>46347</v>
+        <v>160</v>
+      </c>
+      <c r="H19" s="2">
+        <v>46358</v>
       </c>
       <c r="I19">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>171</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>195</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>196</v>
       </c>
       <c r="D20" s="2">
-        <v>45990</v>
-      </c>
-      <c r="F20" t="s">
-        <v>32</v>
-      </c>
-      <c r="H20" s="4">
-        <v>46354</v>
+        <v>45998</v>
+      </c>
+      <c r="E20" t="s">
+        <v>9</v>
+      </c>
+      <c r="H20" s="2">
+        <v>46362</v>
       </c>
       <c r="I20">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -2918,45 +2886,45 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>159</v>
+        <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="D21" s="2">
-        <v>45994</v>
+        <v>45997</v>
       </c>
       <c r="G21" t="s">
-        <v>161</v>
-      </c>
-      <c r="H21" s="4">
-        <v>46358</v>
+        <v>39</v>
+      </c>
+      <c r="H21" s="2">
+        <v>46371</v>
       </c>
       <c r="I21">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>172</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>196</v>
+        <v>156</v>
       </c>
       <c r="C22" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="D22" s="2">
-        <v>45998</v>
-      </c>
-      <c r="E22" t="s">
-        <v>9</v>
-      </c>
-      <c r="H22" s="4">
-        <v>46362</v>
+        <v>46166</v>
+      </c>
+      <c r="G22" t="s">
+        <v>50</v>
+      </c>
+      <c r="H22" s="2">
+        <v>46371</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -2964,65 +2932,65 @@
         <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>47</v>
+        <v>161</v>
       </c>
       <c r="C23" t="s">
-        <v>48</v>
+        <v>159</v>
       </c>
       <c r="D23" s="2">
-        <v>45997</v>
+        <v>46166</v>
       </c>
       <c r="G23" t="s">
-        <v>39</v>
-      </c>
-      <c r="H23" s="4">
+        <v>15</v>
+      </c>
+      <c r="H23" s="2">
         <v>46371</v>
       </c>
       <c r="I23">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="B24" t="s">
-        <v>157</v>
+        <v>74</v>
       </c>
       <c r="C24" t="s">
-        <v>158</v>
+        <v>75</v>
       </c>
       <c r="D24" s="2">
-        <v>46166</v>
+        <v>46041</v>
       </c>
       <c r="G24" t="s">
-        <v>50</v>
-      </c>
-      <c r="H24" s="4">
-        <v>46371</v>
+        <v>39</v>
+      </c>
+      <c r="H24" s="2">
+        <v>46405</v>
       </c>
       <c r="I24">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>170</v>
       </c>
       <c r="B25" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="C25" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="D25" s="2">
-        <v>46166</v>
-      </c>
-      <c r="G25" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" s="4">
-        <v>46371</v>
+        <v>46053</v>
+      </c>
+      <c r="E25" t="s">
+        <v>9</v>
+      </c>
+      <c r="H25" s="2">
+        <v>46417</v>
       </c>
       <c r="I25">
         <v>3</v>
@@ -3030,68 +2998,68 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>170</v>
       </c>
       <c r="B26" t="s">
-        <v>74</v>
+        <v>178</v>
       </c>
       <c r="C26" t="s">
-        <v>75</v>
+        <v>180</v>
       </c>
       <c r="D26" s="2">
-        <v>46041</v>
-      </c>
-      <c r="G26" t="s">
-        <v>39</v>
-      </c>
-      <c r="H26" s="4">
-        <v>46405</v>
+        <v>46054</v>
+      </c>
+      <c r="E26" t="s">
+        <v>9</v>
+      </c>
+      <c r="H26" s="2">
+        <v>46418</v>
       </c>
       <c r="I26">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>171</v>
+        <v>41</v>
       </c>
       <c r="B27" t="s">
-        <v>180</v>
+        <v>68</v>
       </c>
       <c r="C27" t="s">
-        <v>182</v>
+        <v>43</v>
       </c>
       <c r="D27" s="2">
-        <v>46053</v>
+        <v>45690</v>
       </c>
       <c r="E27" t="s">
         <v>9</v>
       </c>
-      <c r="H27" s="4">
-        <v>46417</v>
+      <c r="H27" s="2">
+        <v>46418</v>
       </c>
       <c r="I27">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>171</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>179</v>
+        <v>28</v>
       </c>
       <c r="C28" t="s">
-        <v>181</v>
+        <v>29</v>
       </c>
       <c r="D28" s="2">
-        <v>46054</v>
+        <v>45332</v>
       </c>
       <c r="E28" t="s">
-        <v>9</v>
-      </c>
-      <c r="H28" s="4">
-        <v>46418</v>
+        <v>30</v>
+      </c>
+      <c r="H28" s="2">
+        <v>46423</v>
       </c>
       <c r="I28">
         <v>3</v>
@@ -3099,45 +3067,48 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C29" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="D29" s="2">
-        <v>45690</v>
-      </c>
-      <c r="E29" t="s">
-        <v>9</v>
-      </c>
-      <c r="H29" s="4">
-        <v>46418</v>
+        <v>46061</v>
+      </c>
+      <c r="G29" t="s">
+        <v>39</v>
+      </c>
+      <c r="H29" s="2">
+        <v>46425</v>
       </c>
       <c r="I29">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B30" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="C30" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="D30" s="2">
-        <v>45332</v>
+        <v>46095</v>
       </c>
       <c r="E30" t="s">
-        <v>30</v>
-      </c>
-      <c r="H30" s="4">
-        <v>46423</v>
+        <v>37</v>
+      </c>
+      <c r="G30" t="s">
+        <v>46</v>
+      </c>
+      <c r="H30" s="2">
+        <v>46459</v>
       </c>
       <c r="I30">
         <v>3</v>
@@ -3145,48 +3116,45 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>169</v>
       </c>
       <c r="B31" t="s">
-        <v>72</v>
+        <v>175</v>
       </c>
       <c r="C31" t="s">
-        <v>73</v>
+        <v>176</v>
       </c>
       <c r="D31" s="2">
-        <v>46061</v>
-      </c>
-      <c r="G31" t="s">
-        <v>39</v>
-      </c>
-      <c r="H31" s="4">
-        <v>46425</v>
+        <v>46124</v>
+      </c>
+      <c r="E31" t="s">
+        <v>9</v>
+      </c>
+      <c r="H31" s="2">
+        <v>46478</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B32" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="C32" t="s">
-        <v>46</v>
+        <v>114</v>
       </c>
       <c r="D32" s="2">
-        <v>46095</v>
-      </c>
-      <c r="E32" t="s">
-        <v>37</v>
+        <v>46118</v>
       </c>
       <c r="G32" t="s">
-        <v>46</v>
-      </c>
-      <c r="H32" s="4">
-        <v>46459</v>
+        <v>39</v>
+      </c>
+      <c r="H32" s="2">
+        <v>46478</v>
       </c>
       <c r="I32">
         <v>3</v>
@@ -3194,67 +3162,67 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>170</v>
+        <v>13</v>
       </c>
       <c r="B33" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
       <c r="C33" t="s">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="D33" s="2">
-        <v>46124</v>
+        <v>46137</v>
       </c>
       <c r="E33" t="s">
-        <v>9</v>
-      </c>
-      <c r="H33" s="4">
+        <v>30</v>
+      </c>
+      <c r="H33" s="2">
         <v>46478</v>
       </c>
       <c r="I33">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B34" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C34" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="D34" s="2">
-        <v>46118</v>
+        <v>46134</v>
       </c>
       <c r="G34" t="s">
-        <v>39</v>
-      </c>
-      <c r="H34" s="4">
+        <v>18</v>
+      </c>
+      <c r="H34" s="2">
         <v>46478</v>
       </c>
       <c r="I34">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B35" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="C35" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D35" s="2">
-        <v>46137</v>
-      </c>
-      <c r="E35" t="s">
-        <v>30</v>
-      </c>
-      <c r="H35" s="4">
+        <v>46123</v>
+      </c>
+      <c r="G35" t="s">
+        <v>39</v>
+      </c>
+      <c r="H35" s="2">
         <v>46478</v>
       </c>
       <c r="I35">
@@ -3263,21 +3231,21 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B36" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="C36" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="D36" s="2">
-        <v>46134</v>
+        <v>46117</v>
       </c>
       <c r="G36" t="s">
-        <v>18</v>
-      </c>
-      <c r="H36" s="4">
+        <v>96</v>
+      </c>
+      <c r="H36" s="2">
         <v>46478</v>
       </c>
       <c r="I36">
@@ -3286,21 +3254,21 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>6</v>
+        <v>120</v>
       </c>
       <c r="B37" t="s">
-        <v>145</v>
+        <v>121</v>
       </c>
       <c r="C37" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="D37" s="2">
-        <v>46123</v>
+        <v>46117</v>
       </c>
       <c r="G37" t="s">
         <v>39</v>
       </c>
-      <c r="H37" s="4">
+      <c r="H37" s="2">
         <v>46478</v>
       </c>
       <c r="I37">
@@ -3309,22 +3277,22 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="B38" t="s">
-        <v>94</v>
+        <v>141</v>
       </c>
       <c r="C38" t="s">
-        <v>95</v>
+        <v>142</v>
       </c>
       <c r="D38" s="2">
-        <v>46117</v>
+        <v>46148</v>
       </c>
       <c r="G38" t="s">
-        <v>96</v>
-      </c>
-      <c r="H38" s="4">
-        <v>46478</v>
+        <v>70</v>
+      </c>
+      <c r="H38" s="2">
+        <v>46508</v>
       </c>
       <c r="I38">
         <v>4</v>
@@ -3332,22 +3300,22 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="B39" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="C39" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="D39" s="2">
-        <v>46117</v>
+        <v>46148</v>
       </c>
       <c r="G39" t="s">
-        <v>39</v>
-      </c>
-      <c r="H39" s="4">
-        <v>46478</v>
+        <v>55</v>
+      </c>
+      <c r="H39" s="2">
+        <v>46508</v>
       </c>
       <c r="I39">
         <v>4</v>
@@ -3355,22 +3323,22 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>169</v>
       </c>
       <c r="B40" t="s">
-        <v>141</v>
+        <v>174</v>
       </c>
       <c r="C40" t="s">
-        <v>142</v>
+        <v>177</v>
       </c>
       <c r="D40" s="2">
-        <v>46148</v>
-      </c>
-      <c r="G40" t="s">
-        <v>70</v>
-      </c>
-      <c r="H40" s="4">
-        <v>46508</v>
+        <v>46159</v>
+      </c>
+      <c r="E40" t="s">
+        <v>9</v>
+      </c>
+      <c r="H40" s="2">
+        <v>46523</v>
       </c>
       <c r="I40">
         <v>4</v>
@@ -3378,48 +3346,48 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="D41" s="2">
-        <v>46148</v>
+        <v>46152</v>
       </c>
       <c r="G41" t="s">
-        <v>55</v>
-      </c>
-      <c r="H41" s="4">
-        <v>46508</v>
+        <v>18</v>
+      </c>
+      <c r="H41" s="2">
+        <v>46527</v>
       </c>
       <c r="I41">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>170</v>
+        <v>13</v>
       </c>
       <c r="B42" t="s">
-        <v>175</v>
+        <v>89</v>
       </c>
       <c r="C42" t="s">
-        <v>178</v>
+        <v>90</v>
       </c>
       <c r="D42" s="2">
-        <v>46159</v>
-      </c>
-      <c r="E42" t="s">
-        <v>9</v>
-      </c>
-      <c r="H42" s="4">
-        <v>46523</v>
+        <v>46145</v>
+      </c>
+      <c r="G42" t="s">
+        <v>70</v>
+      </c>
+      <c r="H42" s="2">
+        <v>46527</v>
       </c>
       <c r="I42">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -3427,64 +3395,64 @@
         <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C43" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="D43" s="2">
-        <v>46152</v>
+        <v>46155</v>
       </c>
       <c r="G43" t="s">
-        <v>18</v>
-      </c>
-      <c r="H43" s="4">
+        <v>46</v>
+      </c>
+      <c r="H43" s="2">
         <v>46527</v>
       </c>
       <c r="I43">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B44" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="C44" t="s">
-        <v>90</v>
+        <v>116</v>
       </c>
       <c r="D44" s="2">
-        <v>46145</v>
-      </c>
-      <c r="G44" t="s">
-        <v>70</v>
-      </c>
-      <c r="H44" s="4">
+        <v>46166</v>
+      </c>
+      <c r="F44" t="s">
+        <v>37</v>
+      </c>
+      <c r="H44" s="2">
         <v>46527</v>
       </c>
       <c r="I44">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>137</v>
       </c>
       <c r="C45" t="s">
-        <v>80</v>
+        <v>138</v>
       </c>
       <c r="D45" s="2">
-        <v>46155</v>
-      </c>
-      <c r="G45" t="s">
-        <v>46</v>
-      </c>
-      <c r="H45" s="4">
+        <v>46165</v>
+      </c>
+      <c r="F45" t="s">
+        <v>37</v>
+      </c>
+      <c r="H45" s="2">
         <v>46527</v>
       </c>
       <c r="I45">
@@ -3493,21 +3461,21 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B46" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="C46" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="D46" s="2">
-        <v>46166</v>
+        <v>46165</v>
       </c>
       <c r="F46" t="s">
         <v>37</v>
       </c>
-      <c r="H46" s="4">
+      <c r="H46" s="2">
         <v>46527</v>
       </c>
       <c r="I46">
@@ -3516,67 +3484,67 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B47" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
       <c r="D47" s="2">
-        <v>46165</v>
-      </c>
-      <c r="F47" t="s">
-        <v>37</v>
-      </c>
-      <c r="H47" s="4">
+        <v>46172</v>
+      </c>
+      <c r="E47" t="s">
+        <v>51</v>
+      </c>
+      <c r="H47" s="2">
         <v>46527</v>
       </c>
       <c r="I47">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B48" t="s">
-        <v>106</v>
+        <v>149</v>
       </c>
       <c r="C48" t="s">
-        <v>107</v>
+        <v>153</v>
       </c>
       <c r="D48" s="2">
-        <v>46165</v>
-      </c>
-      <c r="F48" t="s">
-        <v>37</v>
-      </c>
-      <c r="H48" s="4">
+        <v>46166</v>
+      </c>
+      <c r="E48" t="s">
+        <v>105</v>
+      </c>
+      <c r="H48" s="2">
         <v>46527</v>
       </c>
       <c r="I48">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="C49" t="s">
-        <v>155</v>
+        <v>129</v>
       </c>
       <c r="D49" s="2">
-        <v>46172</v>
-      </c>
-      <c r="E49" t="s">
-        <v>51</v>
-      </c>
-      <c r="H49" s="4">
+        <v>46163</v>
+      </c>
+      <c r="G49" t="s">
+        <v>130</v>
+      </c>
+      <c r="H49" s="2">
         <v>46527</v>
       </c>
       <c r="I49">
@@ -3588,42 +3556,42 @@
         <v>13</v>
       </c>
       <c r="B50" t="s">
-        <v>150</v>
+        <v>91</v>
       </c>
       <c r="C50" t="s">
-        <v>154</v>
+        <v>92</v>
       </c>
       <c r="D50" s="2">
-        <v>46166</v>
-      </c>
-      <c r="E50" t="s">
-        <v>105</v>
-      </c>
-      <c r="H50" s="4">
-        <v>46527</v>
+        <v>46131</v>
+      </c>
+      <c r="G50" t="s">
+        <v>21</v>
+      </c>
+      <c r="H50" s="2">
+        <v>46529</v>
       </c>
       <c r="I50">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B51" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="C51" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="D51" s="2">
-        <v>46163</v>
+        <v>46158</v>
       </c>
       <c r="G51" t="s">
-        <v>130</v>
-      </c>
-      <c r="H51" s="4">
-        <v>46527</v>
+        <v>102</v>
+      </c>
+      <c r="H51" s="2">
+        <v>46537</v>
       </c>
       <c r="I51">
         <v>4</v>
@@ -3634,22 +3602,22 @@
         <v>13</v>
       </c>
       <c r="B52" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C52" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D52" s="2">
-        <v>46131</v>
+        <v>46144</v>
       </c>
       <c r="G52" t="s">
-        <v>21</v>
-      </c>
-      <c r="H52" s="4">
-        <v>46529</v>
+        <v>99</v>
+      </c>
+      <c r="H52" s="2">
+        <v>46537</v>
       </c>
       <c r="I52">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -3657,42 +3625,42 @@
         <v>13</v>
       </c>
       <c r="B53" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="C53" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="D53" s="2">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="G53" t="s">
-        <v>102</v>
-      </c>
-      <c r="H53" s="4">
+        <v>55</v>
+      </c>
+      <c r="H53" s="2">
         <v>46537</v>
       </c>
       <c r="I53">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B54" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="C54" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="D54" s="2">
-        <v>46144</v>
+        <v>46178</v>
       </c>
       <c r="G54" t="s">
-        <v>99</v>
-      </c>
-      <c r="H54" s="4">
-        <v>46537</v>
+        <v>119</v>
+      </c>
+      <c r="H54" s="2">
+        <v>46542</v>
       </c>
       <c r="I54">
         <v>4</v>
@@ -3700,229 +3668,229 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>170</v>
       </c>
       <c r="B55" t="s">
-        <v>85</v>
+        <v>191</v>
       </c>
       <c r="C55" t="s">
-        <v>86</v>
+        <v>186</v>
       </c>
       <c r="D55" s="2">
-        <v>46161</v>
-      </c>
-      <c r="G55" t="s">
-        <v>55</v>
-      </c>
-      <c r="H55" s="4">
-        <v>46537</v>
+        <v>46179</v>
+      </c>
+      <c r="E55" t="s">
+        <v>9</v>
+      </c>
+      <c r="H55" s="2">
+        <v>46543</v>
       </c>
       <c r="I55">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B56" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="C56" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="D56" s="2">
-        <v>46178</v>
+        <v>46173</v>
       </c>
       <c r="G56" t="s">
-        <v>119</v>
-      </c>
-      <c r="H56" s="4">
-        <v>46542</v>
+        <v>133</v>
+      </c>
+      <c r="H56" s="2">
+        <v>46543</v>
       </c>
       <c r="I56">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>171</v>
+        <v>13</v>
       </c>
       <c r="B57" t="s">
-        <v>192</v>
+        <v>79</v>
       </c>
       <c r="C57" t="s">
-        <v>187</v>
+        <v>80</v>
       </c>
       <c r="D57" s="2">
-        <v>46179</v>
-      </c>
-      <c r="E57" t="s">
-        <v>9</v>
-      </c>
-      <c r="H57" s="4">
+        <v>46172</v>
+      </c>
+      <c r="F57" t="s">
+        <v>37</v>
+      </c>
+      <c r="H57" s="2">
         <v>46543</v>
       </c>
       <c r="I57">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>22</v>
+        <v>170</v>
       </c>
       <c r="B58" t="s">
-        <v>131</v>
+        <v>188</v>
       </c>
       <c r="C58" t="s">
-        <v>132</v>
+        <v>187</v>
       </c>
       <c r="D58" s="2">
-        <v>46173</v>
-      </c>
-      <c r="G58" t="s">
-        <v>133</v>
-      </c>
-      <c r="H58" s="4">
-        <v>46543</v>
+        <v>46180</v>
+      </c>
+      <c r="E58" t="s">
+        <v>9</v>
+      </c>
+      <c r="H58" s="2">
+        <v>46544</v>
       </c>
       <c r="I58">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="B59" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
       <c r="C59" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="D59" s="2">
-        <v>46172</v>
-      </c>
-      <c r="F59" t="s">
-        <v>37</v>
-      </c>
-      <c r="H59" s="4">
-        <v>46543</v>
+        <v>46180</v>
+      </c>
+      <c r="G59" t="s">
+        <v>21</v>
+      </c>
+      <c r="H59" s="2">
+        <v>46544</v>
       </c>
       <c r="I59">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>171</v>
+        <v>19</v>
       </c>
       <c r="B60" t="s">
-        <v>189</v>
+        <v>111</v>
       </c>
       <c r="C60" t="s">
-        <v>188</v>
+        <v>112</v>
       </c>
       <c r="D60" s="2">
-        <v>46180</v>
-      </c>
-      <c r="E60" t="s">
-        <v>9</v>
-      </c>
-      <c r="H60" s="4">
-        <v>46544</v>
+        <v>46186</v>
+      </c>
+      <c r="G60" t="s">
+        <v>39</v>
+      </c>
+      <c r="H60" s="2">
+        <v>46553</v>
       </c>
       <c r="I60">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="B61" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C61" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="D61" s="2">
-        <v>46180</v>
+        <v>46187</v>
       </c>
       <c r="G61" t="s">
-        <v>21</v>
-      </c>
-      <c r="H61" s="4">
-        <v>46544</v>
+        <v>39</v>
+      </c>
+      <c r="H61" s="2">
+        <v>46553</v>
       </c>
       <c r="I61">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B62" t="s">
-        <v>111</v>
+        <v>144</v>
       </c>
       <c r="C62" t="s">
-        <v>112</v>
+        <v>197</v>
       </c>
       <c r="D62" s="2">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="G62" t="s">
-        <v>39</v>
-      </c>
-      <c r="H62" s="4">
-        <v>46553</v>
+        <v>55</v>
+      </c>
+      <c r="H62" s="2">
+        <v>46557</v>
       </c>
       <c r="I62">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="B63" t="s">
-        <v>125</v>
+        <v>182</v>
       </c>
       <c r="C63" t="s">
-        <v>126</v>
+        <v>199</v>
       </c>
       <c r="D63" s="2">
-        <v>46187</v>
-      </c>
-      <c r="G63" t="s">
-        <v>39</v>
-      </c>
-      <c r="H63" s="4">
-        <v>46553</v>
+        <v>46194</v>
+      </c>
+      <c r="E63" t="s">
+        <v>9</v>
+      </c>
+      <c r="H63" s="2">
+        <v>46558</v>
       </c>
       <c r="I63">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="B64" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C64" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D64" s="2">
-        <v>46193</v>
+        <v>46195</v>
       </c>
       <c r="G64" t="s">
-        <v>55</v>
-      </c>
-      <c r="H64" s="4">
-        <v>46557</v>
+        <v>39</v>
+      </c>
+      <c r="H64" s="2">
+        <v>46559</v>
       </c>
       <c r="I64">
         <v>4</v>
@@ -3938,13 +3906,13 @@
       <c r="C65" t="s">
         <v>27</v>
       </c>
-      <c r="D65" s="4">
+      <c r="D65" s="2">
         <v>45822</v>
       </c>
       <c r="E65" t="s">
         <v>9</v>
       </c>
-      <c r="H65" s="4">
+      <c r="H65" s="2">
         <v>46560</v>
       </c>
       <c r="I65">
@@ -3967,7 +3935,7 @@
       <c r="E66" t="s">
         <v>51</v>
       </c>
-      <c r="H66" s="4">
+      <c r="H66" s="2">
         <v>46569</v>
       </c>
       <c r="I66">
@@ -3990,7 +3958,7 @@
       <c r="E67" t="s">
         <v>105</v>
       </c>
-      <c r="H67" s="4">
+      <c r="H67" s="2">
         <v>46585</v>
       </c>
       <c r="I67">
@@ -4013,7 +3981,7 @@
       <c r="E68" t="s">
         <v>9</v>
       </c>
-      <c r="H68" s="4">
+      <c r="H68" s="2">
         <v>46593</v>
       </c>
       <c r="I68">
@@ -4036,7 +4004,7 @@
       <c r="E69" t="s">
         <v>9</v>
       </c>
-      <c r="H69" s="4">
+      <c r="H69" s="2">
         <v>46631</v>
       </c>
       <c r="I69">
@@ -4059,7 +4027,7 @@
       <c r="E70" t="s">
         <v>9</v>
       </c>
-      <c r="H70" s="4">
+      <c r="H70" s="2">
         <v>46640</v>
       </c>
       <c r="I70">
@@ -4082,7 +4050,7 @@
       <c r="E71" t="s">
         <v>9</v>
       </c>
-      <c r="H71" s="4">
+      <c r="H71" s="2">
         <v>46658</v>
       </c>
       <c r="I71">
@@ -4105,7 +4073,7 @@
       <c r="E72" t="s">
         <v>9</v>
       </c>
-      <c r="H72" s="4">
+      <c r="H72" s="2">
         <v>46704</v>
       </c>
       <c r="I72">
@@ -4128,7 +4096,7 @@
       <c r="E73" t="s">
         <v>9</v>
       </c>
-      <c r="H73" s="4">
+      <c r="H73" s="2">
         <v>46712</v>
       </c>
       <c r="I73">
@@ -4151,7 +4119,7 @@
       <c r="E74" t="s">
         <v>35</v>
       </c>
-      <c r="H74" s="4">
+      <c r="H74" s="2">
         <v>46934</v>
       </c>
       <c r="I74">
@@ -4174,7 +4142,7 @@
       <c r="E75" t="s">
         <v>37</v>
       </c>
-      <c r="H75" s="4">
+      <c r="H75" s="2">
         <v>46948</v>
       </c>
       <c r="I75">
@@ -4197,7 +4165,7 @@
       <c r="E76" t="s">
         <v>32</v>
       </c>
-      <c r="H76" s="4">
+      <c r="H76" s="2">
         <v>46948</v>
       </c>
       <c r="I76">
@@ -4206,10 +4174,10 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B77" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C77" t="s">
         <v>39</v>
@@ -4220,7 +4188,7 @@
       <c r="E77" t="s">
         <v>9</v>
       </c>
-      <c r="H77" s="4">
+      <c r="H77" s="2">
         <v>46964</v>
       </c>
       <c r="I77">
@@ -4243,7 +4211,7 @@
       <c r="E78" t="s">
         <v>9</v>
       </c>
-      <c r="H78" s="4">
+      <c r="H78" s="2">
         <v>46964</v>
       </c>
       <c r="I78">
@@ -4266,7 +4234,7 @@
       <c r="E79" t="s">
         <v>9</v>
       </c>
-      <c r="H79" s="4">
+      <c r="H79" s="2">
         <v>46964</v>
       </c>
       <c r="I79">
@@ -4278,7 +4246,7 @@
         <v>120</v>
       </c>
       <c r="B80" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C80" t="s">
         <v>39</v>
@@ -4289,7 +4257,7 @@
       <c r="E80" t="s">
         <v>9</v>
       </c>
-      <c r="H80" s="4">
+      <c r="H80" s="2">
         <v>46964</v>
       </c>
       <c r="I80">
@@ -4312,7 +4280,7 @@
       <c r="E81" t="s">
         <v>9</v>
       </c>
-      <c r="H81" s="4">
+      <c r="H81" s="2">
         <v>46964</v>
       </c>
       <c r="I81">
@@ -4335,7 +4303,7 @@
       <c r="E82" t="s">
         <v>9</v>
       </c>
-      <c r="H82" s="4">
+      <c r="H82" s="2">
         <v>46964</v>
       </c>
       <c r="I82">
@@ -4358,7 +4326,7 @@
       <c r="E83" t="s">
         <v>9</v>
       </c>
-      <c r="H83" s="4">
+      <c r="H83" s="2">
         <v>47076</v>
       </c>
       <c r="I83">
@@ -4381,7 +4349,7 @@
       <c r="E84" t="s">
         <v>9</v>
       </c>
-      <c r="H84" s="4">
+      <c r="H84" s="2">
         <v>47194</v>
       </c>
       <c r="I84">
@@ -4404,7 +4372,7 @@
       <c r="F85" t="s">
         <v>9</v>
       </c>
-      <c r="H85" s="4">
+      <c r="H85" s="2">
         <v>47316</v>
       </c>
       <c r="I85">
@@ -4427,7 +4395,7 @@
       <c r="E86" t="s">
         <v>37</v>
       </c>
-      <c r="H86" s="4">
+      <c r="H86" s="2">
         <v>47325</v>
       </c>
       <c r="I86">
@@ -4436,13 +4404,13 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>164</v>
+      </c>
+      <c r="B87" t="s">
+        <v>162</v>
+      </c>
+      <c r="C87" t="s">
         <v>165</v>
-      </c>
-      <c r="B87" t="s">
-        <v>163</v>
-      </c>
-      <c r="C87" t="s">
-        <v>166</v>
       </c>
       <c r="D87" s="2">
         <v>46075</v>
@@ -4450,7 +4418,7 @@
       <c r="E87" t="s">
         <v>9</v>
       </c>
-      <c r="H87" s="4">
+      <c r="H87" s="2">
         <v>47536</v>
       </c>
       <c r="I87">
@@ -4473,7 +4441,7 @@
       <c r="E88" t="s">
         <v>9</v>
       </c>
-      <c r="H88" s="4">
+      <c r="H88" s="2">
         <v>47536</v>
       </c>
       <c r="I88">

</xml_diff>